<commit_message>
feat(buyer-unit-details): regenerate TCs APPROVED — 19 TCs, 94.7% coverage
Prior TCs were STUB-based (Conditional). INDEX.md updated to FULL after
WINNER account (GHNG-1000008364-C) captured the real feature: unit details
is a PDF download button on the KYC success page (/kyc?unitId=<b64>),
not a separate /allotted-units route (all direct URLs 404).

DOC_DRIFT-001 flagged: FRD URL header obsolete — will fix in next sync Step 2.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/manual-qa-repository/07-execution/TestCases-Consolidated.xlsx
+++ b/manual-qa-repository/07-execution/TestCases-Consolidated.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17382" uniqueCount="5292">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17686" uniqueCount="5313">
   <si>
     <t>TC ID</t>
   </si>
@@ -16545,6 +16545,69 @@
   </si>
   <si>
     <t>TC_PHYSALLOC_UI_055</t>
+  </si>
+  <si>
+    <t>TC_BUYUD_NEG_001</t>
+  </si>
+  <si>
+    <t>FULL</t>
+  </si>
+  <si>
+    <t>TC_BUYUD_NEG_002</t>
+  </si>
+  <si>
+    <t>TC_BUYUD_FUNC_001</t>
+  </si>
+  <si>
+    <t>TC_BUYUD_FUNC_002</t>
+  </si>
+  <si>
+    <t>TC_BUYUD_FUNC_003</t>
+  </si>
+  <si>
+    <t>TC_BUYUD_VAL_001</t>
+  </si>
+  <si>
+    <t>TC_BUYUD_FUNC_004</t>
+  </si>
+  <si>
+    <t>TC_BUYUD_FUNC_005</t>
+  </si>
+  <si>
+    <t>TC_BUYUD_FUNC_006</t>
+  </si>
+  <si>
+    <t>TC_BUYUD_FUNC_007</t>
+  </si>
+  <si>
+    <t>TC_BUYUD_FUNC_008</t>
+  </si>
+  <si>
+    <t>TC_BUYUD_BIZ_001</t>
+  </si>
+  <si>
+    <t>TC_BUYUD_NEG_003</t>
+  </si>
+  <si>
+    <t>FULL (negative)</t>
+  </si>
+  <si>
+    <t>TC_BUYUD_NEG_004</t>
+  </si>
+  <si>
+    <t>TC_BUYUD_UI_001</t>
+  </si>
+  <si>
+    <t>TC_BUYUD_UI_002</t>
+  </si>
+  <si>
+    <t>TC_BUYUD_REG_001</t>
+  </si>
+  <si>
+    <t>TC_BUYUD_XMOD_001</t>
+  </si>
+  <si>
+    <t>TC_BUYUD_EDGE_001</t>
   </si>
   <si>
     <t>Total TCs</t>
@@ -17167,7 +17230,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:P1092"/>
+  <dimension ref="A1:P1111"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="24" customWidth="1"/>
@@ -71485,6 +71548,956 @@
       </c>
       <c r="P1092" t="s">
         <v>30</v>
+      </c>
+    </row>
+    <row r="1093" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A1093" t="s">
+        <v>5284</v>
+      </c>
+      <c r="B1093" t="s">
+        <v>1650</v>
+      </c>
+      <c r="C1093" t="s">
+        <v>2670</v>
+      </c>
+      <c r="D1093" t="s">
+        <v>148</v>
+      </c>
+      <c r="E1093" t="s">
+        <v>30</v>
+      </c>
+      <c r="F1093" t="s">
+        <v>30</v>
+      </c>
+      <c r="G1093" t="s">
+        <v>30</v>
+      </c>
+      <c r="H1093" t="s">
+        <v>30</v>
+      </c>
+      <c r="I1093" t="s">
+        <v>30</v>
+      </c>
+      <c r="J1093" t="s">
+        <v>26</v>
+      </c>
+      <c r="K1093" t="s">
+        <v>30</v>
+      </c>
+      <c r="L1093" t="s">
+        <v>30</v>
+      </c>
+      <c r="M1093" t="s">
+        <v>1657</v>
+      </c>
+      <c r="N1093" t="s">
+        <v>30</v>
+      </c>
+      <c r="O1093" t="s">
+        <v>30</v>
+      </c>
+      <c r="P1093" t="s">
+        <v>5285</v>
+      </c>
+    </row>
+    <row r="1094" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A1094" t="s">
+        <v>5286</v>
+      </c>
+      <c r="B1094" t="s">
+        <v>1650</v>
+      </c>
+      <c r="C1094" t="s">
+        <v>2670</v>
+      </c>
+      <c r="D1094" t="s">
+        <v>148</v>
+      </c>
+      <c r="E1094" t="s">
+        <v>30</v>
+      </c>
+      <c r="F1094" t="s">
+        <v>30</v>
+      </c>
+      <c r="G1094" t="s">
+        <v>30</v>
+      </c>
+      <c r="H1094" t="s">
+        <v>30</v>
+      </c>
+      <c r="I1094" t="s">
+        <v>30</v>
+      </c>
+      <c r="J1094" t="s">
+        <v>26</v>
+      </c>
+      <c r="K1094" t="s">
+        <v>30</v>
+      </c>
+      <c r="L1094" t="s">
+        <v>30</v>
+      </c>
+      <c r="M1094" t="s">
+        <v>1657</v>
+      </c>
+      <c r="N1094" t="s">
+        <v>30</v>
+      </c>
+      <c r="O1094" t="s">
+        <v>30</v>
+      </c>
+      <c r="P1094" t="s">
+        <v>5285</v>
+      </c>
+    </row>
+    <row r="1095" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A1095" t="s">
+        <v>5287</v>
+      </c>
+      <c r="B1095" t="s">
+        <v>1650</v>
+      </c>
+      <c r="C1095" t="s">
+        <v>2670</v>
+      </c>
+      <c r="D1095" t="s">
+        <v>53</v>
+      </c>
+      <c r="E1095" t="s">
+        <v>30</v>
+      </c>
+      <c r="F1095" t="s">
+        <v>30</v>
+      </c>
+      <c r="G1095" t="s">
+        <v>30</v>
+      </c>
+      <c r="H1095" t="s">
+        <v>30</v>
+      </c>
+      <c r="I1095" t="s">
+        <v>30</v>
+      </c>
+      <c r="J1095" t="s">
+        <v>26</v>
+      </c>
+      <c r="K1095" t="s">
+        <v>30</v>
+      </c>
+      <c r="L1095" t="s">
+        <v>30</v>
+      </c>
+      <c r="M1095" t="s">
+        <v>1657</v>
+      </c>
+      <c r="N1095" t="s">
+        <v>30</v>
+      </c>
+      <c r="O1095" t="s">
+        <v>30</v>
+      </c>
+      <c r="P1095" t="s">
+        <v>5285</v>
+      </c>
+    </row>
+    <row r="1096" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A1096" t="s">
+        <v>5288</v>
+      </c>
+      <c r="B1096" t="s">
+        <v>1650</v>
+      </c>
+      <c r="C1096" t="s">
+        <v>2670</v>
+      </c>
+      <c r="D1096" t="s">
+        <v>53</v>
+      </c>
+      <c r="E1096" t="s">
+        <v>30</v>
+      </c>
+      <c r="F1096" t="s">
+        <v>30</v>
+      </c>
+      <c r="G1096" t="s">
+        <v>30</v>
+      </c>
+      <c r="H1096" t="s">
+        <v>30</v>
+      </c>
+      <c r="I1096" t="s">
+        <v>30</v>
+      </c>
+      <c r="J1096" t="s">
+        <v>26</v>
+      </c>
+      <c r="K1096" t="s">
+        <v>30</v>
+      </c>
+      <c r="L1096" t="s">
+        <v>30</v>
+      </c>
+      <c r="M1096" t="s">
+        <v>1657</v>
+      </c>
+      <c r="N1096" t="s">
+        <v>30</v>
+      </c>
+      <c r="O1096" t="s">
+        <v>30</v>
+      </c>
+      <c r="P1096" t="s">
+        <v>5285</v>
+      </c>
+    </row>
+    <row r="1097" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A1097" t="s">
+        <v>5289</v>
+      </c>
+      <c r="B1097" t="s">
+        <v>1650</v>
+      </c>
+      <c r="C1097" t="s">
+        <v>2670</v>
+      </c>
+      <c r="D1097" t="s">
+        <v>53</v>
+      </c>
+      <c r="E1097" t="s">
+        <v>30</v>
+      </c>
+      <c r="F1097" t="s">
+        <v>30</v>
+      </c>
+      <c r="G1097" t="s">
+        <v>30</v>
+      </c>
+      <c r="H1097" t="s">
+        <v>30</v>
+      </c>
+      <c r="I1097" t="s">
+        <v>30</v>
+      </c>
+      <c r="J1097" t="s">
+        <v>26</v>
+      </c>
+      <c r="K1097" t="s">
+        <v>30</v>
+      </c>
+      <c r="L1097" t="s">
+        <v>30</v>
+      </c>
+      <c r="M1097" t="s">
+        <v>1657</v>
+      </c>
+      <c r="N1097" t="s">
+        <v>30</v>
+      </c>
+      <c r="O1097" t="s">
+        <v>30</v>
+      </c>
+      <c r="P1097" t="s">
+        <v>5285</v>
+      </c>
+    </row>
+    <row r="1098" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A1098" t="s">
+        <v>5290</v>
+      </c>
+      <c r="B1098" t="s">
+        <v>1650</v>
+      </c>
+      <c r="C1098" t="s">
+        <v>2670</v>
+      </c>
+      <c r="D1098" t="s">
+        <v>119</v>
+      </c>
+      <c r="E1098" t="s">
+        <v>30</v>
+      </c>
+      <c r="F1098" t="s">
+        <v>30</v>
+      </c>
+      <c r="G1098" t="s">
+        <v>30</v>
+      </c>
+      <c r="H1098" t="s">
+        <v>30</v>
+      </c>
+      <c r="I1098" t="s">
+        <v>30</v>
+      </c>
+      <c r="J1098" t="s">
+        <v>26</v>
+      </c>
+      <c r="K1098" t="s">
+        <v>30</v>
+      </c>
+      <c r="L1098" t="s">
+        <v>30</v>
+      </c>
+      <c r="M1098" t="s">
+        <v>1657</v>
+      </c>
+      <c r="N1098" t="s">
+        <v>30</v>
+      </c>
+      <c r="O1098" t="s">
+        <v>30</v>
+      </c>
+      <c r="P1098" t="s">
+        <v>5285</v>
+      </c>
+    </row>
+    <row r="1099" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A1099" t="s">
+        <v>5291</v>
+      </c>
+      <c r="B1099" t="s">
+        <v>1650</v>
+      </c>
+      <c r="C1099" t="s">
+        <v>2670</v>
+      </c>
+      <c r="D1099" t="s">
+        <v>53</v>
+      </c>
+      <c r="E1099" t="s">
+        <v>30</v>
+      </c>
+      <c r="F1099" t="s">
+        <v>30</v>
+      </c>
+      <c r="G1099" t="s">
+        <v>30</v>
+      </c>
+      <c r="H1099" t="s">
+        <v>30</v>
+      </c>
+      <c r="I1099" t="s">
+        <v>30</v>
+      </c>
+      <c r="J1099" t="s">
+        <v>26</v>
+      </c>
+      <c r="K1099" t="s">
+        <v>30</v>
+      </c>
+      <c r="L1099" t="s">
+        <v>30</v>
+      </c>
+      <c r="M1099" t="s">
+        <v>1657</v>
+      </c>
+      <c r="N1099" t="s">
+        <v>30</v>
+      </c>
+      <c r="O1099" t="s">
+        <v>30</v>
+      </c>
+      <c r="P1099" t="s">
+        <v>5285</v>
+      </c>
+    </row>
+    <row r="1100" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A1100" t="s">
+        <v>5292</v>
+      </c>
+      <c r="B1100" t="s">
+        <v>1650</v>
+      </c>
+      <c r="C1100" t="s">
+        <v>2670</v>
+      </c>
+      <c r="D1100" t="s">
+        <v>53</v>
+      </c>
+      <c r="E1100" t="s">
+        <v>30</v>
+      </c>
+      <c r="F1100" t="s">
+        <v>30</v>
+      </c>
+      <c r="G1100" t="s">
+        <v>30</v>
+      </c>
+      <c r="H1100" t="s">
+        <v>30</v>
+      </c>
+      <c r="I1100" t="s">
+        <v>30</v>
+      </c>
+      <c r="J1100" t="s">
+        <v>26</v>
+      </c>
+      <c r="K1100" t="s">
+        <v>30</v>
+      </c>
+      <c r="L1100" t="s">
+        <v>30</v>
+      </c>
+      <c r="M1100" t="s">
+        <v>1657</v>
+      </c>
+      <c r="N1100" t="s">
+        <v>30</v>
+      </c>
+      <c r="O1100" t="s">
+        <v>30</v>
+      </c>
+      <c r="P1100" t="s">
+        <v>5285</v>
+      </c>
+    </row>
+    <row r="1101" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A1101" t="s">
+        <v>5293</v>
+      </c>
+      <c r="B1101" t="s">
+        <v>1650</v>
+      </c>
+      <c r="C1101" t="s">
+        <v>2670</v>
+      </c>
+      <c r="D1101" t="s">
+        <v>53</v>
+      </c>
+      <c r="E1101" t="s">
+        <v>30</v>
+      </c>
+      <c r="F1101" t="s">
+        <v>30</v>
+      </c>
+      <c r="G1101" t="s">
+        <v>30</v>
+      </c>
+      <c r="H1101" t="s">
+        <v>30</v>
+      </c>
+      <c r="I1101" t="s">
+        <v>30</v>
+      </c>
+      <c r="J1101" t="s">
+        <v>26</v>
+      </c>
+      <c r="K1101" t="s">
+        <v>30</v>
+      </c>
+      <c r="L1101" t="s">
+        <v>30</v>
+      </c>
+      <c r="M1101" t="s">
+        <v>1657</v>
+      </c>
+      <c r="N1101" t="s">
+        <v>30</v>
+      </c>
+      <c r="O1101" t="s">
+        <v>30</v>
+      </c>
+      <c r="P1101" t="s">
+        <v>5285</v>
+      </c>
+    </row>
+    <row r="1102" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A1102" t="s">
+        <v>5294</v>
+      </c>
+      <c r="B1102" t="s">
+        <v>1650</v>
+      </c>
+      <c r="C1102" t="s">
+        <v>2670</v>
+      </c>
+      <c r="D1102" t="s">
+        <v>53</v>
+      </c>
+      <c r="E1102" t="s">
+        <v>30</v>
+      </c>
+      <c r="F1102" t="s">
+        <v>30</v>
+      </c>
+      <c r="G1102" t="s">
+        <v>30</v>
+      </c>
+      <c r="H1102" t="s">
+        <v>30</v>
+      </c>
+      <c r="I1102" t="s">
+        <v>30</v>
+      </c>
+      <c r="J1102" t="s">
+        <v>26</v>
+      </c>
+      <c r="K1102" t="s">
+        <v>30</v>
+      </c>
+      <c r="L1102" t="s">
+        <v>30</v>
+      </c>
+      <c r="M1102" t="s">
+        <v>1657</v>
+      </c>
+      <c r="N1102" t="s">
+        <v>30</v>
+      </c>
+      <c r="O1102" t="s">
+        <v>30</v>
+      </c>
+      <c r="P1102" t="s">
+        <v>5285</v>
+      </c>
+    </row>
+    <row r="1103" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A1103" t="s">
+        <v>5295</v>
+      </c>
+      <c r="B1103" t="s">
+        <v>1650</v>
+      </c>
+      <c r="C1103" t="s">
+        <v>2670</v>
+      </c>
+      <c r="D1103" t="s">
+        <v>53</v>
+      </c>
+      <c r="E1103" t="s">
+        <v>30</v>
+      </c>
+      <c r="F1103" t="s">
+        <v>30</v>
+      </c>
+      <c r="G1103" t="s">
+        <v>30</v>
+      </c>
+      <c r="H1103" t="s">
+        <v>30</v>
+      </c>
+      <c r="I1103" t="s">
+        <v>30</v>
+      </c>
+      <c r="J1103" t="s">
+        <v>26</v>
+      </c>
+      <c r="K1103" t="s">
+        <v>30</v>
+      </c>
+      <c r="L1103" t="s">
+        <v>30</v>
+      </c>
+      <c r="M1103" t="s">
+        <v>1657</v>
+      </c>
+      <c r="N1103" t="s">
+        <v>30</v>
+      </c>
+      <c r="O1103" t="s">
+        <v>30</v>
+      </c>
+      <c r="P1103" t="s">
+        <v>5285</v>
+      </c>
+    </row>
+    <row r="1104" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A1104" t="s">
+        <v>5296</v>
+      </c>
+      <c r="B1104" t="s">
+        <v>1650</v>
+      </c>
+      <c r="C1104" t="s">
+        <v>2670</v>
+      </c>
+      <c r="D1104" t="s">
+        <v>186</v>
+      </c>
+      <c r="E1104" t="s">
+        <v>30</v>
+      </c>
+      <c r="F1104" t="s">
+        <v>30</v>
+      </c>
+      <c r="G1104" t="s">
+        <v>30</v>
+      </c>
+      <c r="H1104" t="s">
+        <v>30</v>
+      </c>
+      <c r="I1104" t="s">
+        <v>30</v>
+      </c>
+      <c r="J1104" t="s">
+        <v>26</v>
+      </c>
+      <c r="K1104" t="s">
+        <v>30</v>
+      </c>
+      <c r="L1104" t="s">
+        <v>30</v>
+      </c>
+      <c r="M1104" t="s">
+        <v>1657</v>
+      </c>
+      <c r="N1104" t="s">
+        <v>30</v>
+      </c>
+      <c r="O1104" t="s">
+        <v>30</v>
+      </c>
+      <c r="P1104" t="s">
+        <v>5285</v>
+      </c>
+    </row>
+    <row r="1105" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A1105" t="s">
+        <v>5297</v>
+      </c>
+      <c r="B1105" t="s">
+        <v>1650</v>
+      </c>
+      <c r="C1105" t="s">
+        <v>2670</v>
+      </c>
+      <c r="D1105" t="s">
+        <v>148</v>
+      </c>
+      <c r="E1105" t="s">
+        <v>30</v>
+      </c>
+      <c r="F1105" t="s">
+        <v>30</v>
+      </c>
+      <c r="G1105" t="s">
+        <v>30</v>
+      </c>
+      <c r="H1105" t="s">
+        <v>30</v>
+      </c>
+      <c r="I1105" t="s">
+        <v>30</v>
+      </c>
+      <c r="J1105" t="s">
+        <v>26</v>
+      </c>
+      <c r="K1105" t="s">
+        <v>30</v>
+      </c>
+      <c r="L1105" t="s">
+        <v>30</v>
+      </c>
+      <c r="M1105" t="s">
+        <v>1657</v>
+      </c>
+      <c r="N1105" t="s">
+        <v>30</v>
+      </c>
+      <c r="O1105" t="s">
+        <v>30</v>
+      </c>
+      <c r="P1105" t="s">
+        <v>5298</v>
+      </c>
+    </row>
+    <row r="1106" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A1106" t="s">
+        <v>5299</v>
+      </c>
+      <c r="B1106" t="s">
+        <v>1650</v>
+      </c>
+      <c r="C1106" t="s">
+        <v>2670</v>
+      </c>
+      <c r="D1106" t="s">
+        <v>148</v>
+      </c>
+      <c r="E1106" t="s">
+        <v>30</v>
+      </c>
+      <c r="F1106" t="s">
+        <v>30</v>
+      </c>
+      <c r="G1106" t="s">
+        <v>30</v>
+      </c>
+      <c r="H1106" t="s">
+        <v>30</v>
+      </c>
+      <c r="I1106" t="s">
+        <v>30</v>
+      </c>
+      <c r="J1106" t="s">
+        <v>26</v>
+      </c>
+      <c r="K1106" t="s">
+        <v>30</v>
+      </c>
+      <c r="L1106" t="s">
+        <v>30</v>
+      </c>
+      <c r="M1106" t="s">
+        <v>1657</v>
+      </c>
+      <c r="N1106" t="s">
+        <v>30</v>
+      </c>
+      <c r="O1106" t="s">
+        <v>30</v>
+      </c>
+      <c r="P1106" t="s">
+        <v>5298</v>
+      </c>
+    </row>
+    <row r="1107" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A1107" t="s">
+        <v>5300</v>
+      </c>
+      <c r="B1107" t="s">
+        <v>1650</v>
+      </c>
+      <c r="C1107" t="s">
+        <v>2670</v>
+      </c>
+      <c r="D1107" t="s">
+        <v>20</v>
+      </c>
+      <c r="E1107" t="s">
+        <v>30</v>
+      </c>
+      <c r="F1107" t="s">
+        <v>30</v>
+      </c>
+      <c r="G1107" t="s">
+        <v>30</v>
+      </c>
+      <c r="H1107" t="s">
+        <v>30</v>
+      </c>
+      <c r="I1107" t="s">
+        <v>30</v>
+      </c>
+      <c r="J1107" t="s">
+        <v>26</v>
+      </c>
+      <c r="K1107" t="s">
+        <v>30</v>
+      </c>
+      <c r="L1107" t="s">
+        <v>30</v>
+      </c>
+      <c r="M1107" t="s">
+        <v>1657</v>
+      </c>
+      <c r="N1107" t="s">
+        <v>30</v>
+      </c>
+      <c r="O1107" t="s">
+        <v>30</v>
+      </c>
+      <c r="P1107" t="s">
+        <v>5285</v>
+      </c>
+    </row>
+    <row r="1108" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A1108" t="s">
+        <v>5301</v>
+      </c>
+      <c r="B1108" t="s">
+        <v>1650</v>
+      </c>
+      <c r="C1108" t="s">
+        <v>2670</v>
+      </c>
+      <c r="D1108" t="s">
+        <v>20</v>
+      </c>
+      <c r="E1108" t="s">
+        <v>30</v>
+      </c>
+      <c r="F1108" t="s">
+        <v>30</v>
+      </c>
+      <c r="G1108" t="s">
+        <v>30</v>
+      </c>
+      <c r="H1108" t="s">
+        <v>30</v>
+      </c>
+      <c r="I1108" t="s">
+        <v>30</v>
+      </c>
+      <c r="J1108" t="s">
+        <v>26</v>
+      </c>
+      <c r="K1108" t="s">
+        <v>30</v>
+      </c>
+      <c r="L1108" t="s">
+        <v>30</v>
+      </c>
+      <c r="M1108" t="s">
+        <v>1657</v>
+      </c>
+      <c r="N1108" t="s">
+        <v>30</v>
+      </c>
+      <c r="O1108" t="s">
+        <v>30</v>
+      </c>
+      <c r="P1108" t="s">
+        <v>5285</v>
+      </c>
+    </row>
+    <row r="1109" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A1109" t="s">
+        <v>5302</v>
+      </c>
+      <c r="B1109" t="s">
+        <v>1650</v>
+      </c>
+      <c r="C1109" t="s">
+        <v>2670</v>
+      </c>
+      <c r="D1109" t="s">
+        <v>749</v>
+      </c>
+      <c r="E1109" t="s">
+        <v>30</v>
+      </c>
+      <c r="F1109" t="s">
+        <v>30</v>
+      </c>
+      <c r="G1109" t="s">
+        <v>30</v>
+      </c>
+      <c r="H1109" t="s">
+        <v>30</v>
+      </c>
+      <c r="I1109" t="s">
+        <v>30</v>
+      </c>
+      <c r="J1109" t="s">
+        <v>26</v>
+      </c>
+      <c r="K1109" t="s">
+        <v>30</v>
+      </c>
+      <c r="L1109" t="s">
+        <v>30</v>
+      </c>
+      <c r="M1109" t="s">
+        <v>1657</v>
+      </c>
+      <c r="N1109" t="s">
+        <v>30</v>
+      </c>
+      <c r="O1109" t="s">
+        <v>30</v>
+      </c>
+      <c r="P1109" t="s">
+        <v>5285</v>
+      </c>
+    </row>
+    <row r="1110" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A1110" t="s">
+        <v>5303</v>
+      </c>
+      <c r="B1110" t="s">
+        <v>1650</v>
+      </c>
+      <c r="C1110" t="s">
+        <v>2670</v>
+      </c>
+      <c r="D1110" t="s">
+        <v>2688</v>
+      </c>
+      <c r="E1110" t="s">
+        <v>30</v>
+      </c>
+      <c r="F1110" t="s">
+        <v>30</v>
+      </c>
+      <c r="G1110" t="s">
+        <v>30</v>
+      </c>
+      <c r="H1110" t="s">
+        <v>30</v>
+      </c>
+      <c r="I1110" t="s">
+        <v>30</v>
+      </c>
+      <c r="J1110" t="s">
+        <v>26</v>
+      </c>
+      <c r="K1110" t="s">
+        <v>30</v>
+      </c>
+      <c r="L1110" t="s">
+        <v>30</v>
+      </c>
+      <c r="M1110" t="s">
+        <v>1657</v>
+      </c>
+      <c r="N1110" t="s">
+        <v>30</v>
+      </c>
+      <c r="O1110" t="s">
+        <v>30</v>
+      </c>
+      <c r="P1110" t="s">
+        <v>5285</v>
+      </c>
+    </row>
+    <row r="1111" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A1111" t="s">
+        <v>5304</v>
+      </c>
+      <c r="B1111" t="s">
+        <v>1650</v>
+      </c>
+      <c r="C1111" t="s">
+        <v>2670</v>
+      </c>
+      <c r="D1111" t="s">
+        <v>170</v>
+      </c>
+      <c r="E1111" t="s">
+        <v>30</v>
+      </c>
+      <c r="F1111" t="s">
+        <v>30</v>
+      </c>
+      <c r="G1111" t="s">
+        <v>30</v>
+      </c>
+      <c r="H1111" t="s">
+        <v>30</v>
+      </c>
+      <c r="I1111" t="s">
+        <v>30</v>
+      </c>
+      <c r="J1111" t="s">
+        <v>26</v>
+      </c>
+      <c r="K1111" t="s">
+        <v>30</v>
+      </c>
+      <c r="L1111" t="s">
+        <v>30</v>
+      </c>
+      <c r="M1111" t="s">
+        <v>1657</v>
+      </c>
+      <c r="N1111" t="s">
+        <v>30</v>
+      </c>
+      <c r="O1111" t="s">
+        <v>30</v>
+      </c>
+      <c r="P1111" t="s">
+        <v>325</v>
       </c>
     </row>
   </sheetData>
@@ -71527,7 +72540,7 @@
         <v>2</v>
       </c>
       <c r="C1" s="32" t="s">
-        <v>5284</v>
+        <v>5305</v>
       </c>
       <c r="D1" s="32" t="s">
         <v>53</v>
@@ -71560,7 +72573,7 @@
         <v>9</v>
       </c>
       <c r="N1" s="32" t="s">
-        <v>5285</v>
+        <v>5306</v>
       </c>
     </row>
     <row r="2" spans="1:14" x14ac:dyDescent="0.25">
@@ -71604,7 +72617,7 @@
         <v>39</v>
       </c>
       <c r="N2" s="34" t="s">
-        <v>5286</v>
+        <v>5307</v>
       </c>
     </row>
     <row r="3" spans="1:14" x14ac:dyDescent="0.25">
@@ -71648,7 +72661,7 @@
         <v>36</v>
       </c>
       <c r="N3" s="36" t="s">
-        <v>5286</v>
+        <v>5307</v>
       </c>
     </row>
     <row r="4" spans="1:14" x14ac:dyDescent="0.25">
@@ -71692,7 +72705,7 @@
         <v>35</v>
       </c>
       <c r="N4" s="34" t="s">
-        <v>5286</v>
+        <v>5307</v>
       </c>
     </row>
     <row r="5" spans="1:14" x14ac:dyDescent="0.25">
@@ -71736,7 +72749,7 @@
         <v>0</v>
       </c>
       <c r="N5" s="36" t="s">
-        <v>5287</v>
+        <v>5308</v>
       </c>
     </row>
     <row r="6" spans="1:14" x14ac:dyDescent="0.25">
@@ -71780,7 +72793,7 @@
         <v>33</v>
       </c>
       <c r="N6" s="34" t="s">
-        <v>5286</v>
+        <v>5307</v>
       </c>
     </row>
     <row r="7" spans="1:14" x14ac:dyDescent="0.25">
@@ -71824,7 +72837,7 @@
         <v>22</v>
       </c>
       <c r="N7" s="36" t="s">
-        <v>5286</v>
+        <v>5307</v>
       </c>
     </row>
     <row r="8" spans="1:14" x14ac:dyDescent="0.25">
@@ -71868,7 +72881,7 @@
         <v>36</v>
       </c>
       <c r="N8" s="34" t="s">
-        <v>5286</v>
+        <v>5307</v>
       </c>
     </row>
     <row r="9" spans="1:14" x14ac:dyDescent="0.25">
@@ -71912,7 +72925,7 @@
         <v>34</v>
       </c>
       <c r="N9" s="36" t="s">
-        <v>5286</v>
+        <v>5307</v>
       </c>
     </row>
     <row r="10" spans="1:14" x14ac:dyDescent="0.25">
@@ -71956,7 +72969,7 @@
         <v>36</v>
       </c>
       <c r="N10" s="34" t="s">
-        <v>5286</v>
+        <v>5307</v>
       </c>
     </row>
     <row r="11" spans="1:14" x14ac:dyDescent="0.25">
@@ -72000,12 +73013,12 @@
         <v>29</v>
       </c>
       <c r="N11" s="36" t="s">
-        <v>5286</v>
+        <v>5307</v>
       </c>
     </row>
     <row r="13" spans="1:14" s="37" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A13" s="37" t="s">
-        <v>5288</v>
+        <v>5309</v>
       </c>
       <c r="B13" s="37" t="s">
         <v>30</v>
@@ -72017,7 +73030,7 @@
         <v>300</v>
       </c>
       <c r="N13" s="37" t="s">
-        <v>5289</v>
+        <v>5310</v>
       </c>
     </row>
   </sheetData>
@@ -72041,7 +73054,7 @@
         <v>3</v>
       </c>
       <c r="B1" s="32" t="s">
-        <v>5290</v>
+        <v>5311</v>
       </c>
       <c r="C1" s="32" t="s">
         <v>9</v>
@@ -72148,7 +73161,7 @@
     </row>
     <row r="12" spans="1:3" s="37" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A12" s="37" t="s">
-        <v>5291</v>
+        <v>5312</v>
       </c>
       <c r="B12" s="37">
         <v>332</v>

</xml_diff>